<commit_message>
feat: add optional Jabatan column, support multi-page printing, and refine recipient management UI
</commit_message>
<xml_diff>
--- a/public/template_impor_labelpro.xlsx
+++ b/public/template_impor_labelpro.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Data Penerima" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -17,22 +17,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="6">
   <si>
-    <t>nama</t>
-  </si>
-  <si>
-    <t>alamat</t>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Jabatan (Opsional)</t>
+  </si>
+  <si>
+    <t>Alamat (Opsional)</t>
   </si>
   <si>
     <t>Budi Santoso</t>
   </si>
   <si>
-    <t>Jl. Melati No. 12, Jakarta</t>
-  </si>
-  <si>
-    <t>Siti Aminah</t>
-  </si>
-  <si>
-    <t>Perumahan Indah Blok C3, Bandung</t>
+    <t>Direktur</t>
+  </si>
+  <si>
+    <t>Jl. Melati No. 10</t>
   </si>
 </sst>
 </file>
@@ -40,7 +40,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -50,28 +50,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF059669"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -86,9 +71,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,34 +372,28 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="38.848" bestFit="true" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>